<commit_message>
feat: add CSV and Excel templates for user import
</commit_message>
<xml_diff>
--- a/frontend/public/Import_Users_Template.xlsx
+++ b/frontend/public/Import_Users_Template.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Users Template" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Template" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="21">
   <si>
     <t>fullname</t>
   </si>
@@ -25,9 +25,6 @@
     <t>role</t>
   </si>
   <si>
-    <t>leader_email</t>
-  </si>
-  <si>
     <t>status</t>
   </si>
   <si>
@@ -52,9 +49,6 @@
     <t>storyboard</t>
   </si>
   <si>
-    <t>leader@company.com</t>
-  </si>
-  <si>
     <t>active</t>
   </si>
   <si>
@@ -70,7 +64,7 @@
     <t>Somsak Rakdee</t>
   </si>
   <si>
-    <t>somsak@example.com</t>
+    <t>somsak@company.com</t>
   </si>
   <si>
     <t>+66898765432</t>
@@ -466,19 +460,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="15" customWidth="1"/>
-    <col min="7" max="9" width="18" customWidth="1"/>
+    <col min="3" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="8" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -503,66 +495,57 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>8</v>
       </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" t="s">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" t="s">
         <v>12</v>
       </c>
-      <c r="E2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="F3" t="s">
         <v>20</v>
       </c>
-      <c r="D3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E3" t="s">
-        <v>22</v>
-      </c>
-      <c r="F3" t="s">
-        <v>14</v>
-      </c>
       <c r="G3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -570,7 +553,7 @@
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Role" error="Please select a role from the dropdown list." sqref="D2:D500">
       <formula1>"admin,manager,storyboard,animation,designer,programmer"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Status" error="Please select a status from the dropdown list." sqref="F2:F500">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid Status" error="Please select a status from the dropdown list." sqref="E2:E500">
       <formula1>"active,suspended"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>